<commit_message>
update(SetupsAI): consolidated website directory (89 unique websites) - 2026-10-25 10:08:04
</commit_message>
<xml_diff>
--- a/📁 SetupsAI/📊 SetupsAI_Websites_Master_List.xlsx
+++ b/📁 SetupsAI/📊 SetupsAI_Websites_Master_List.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:F90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -561,7 +561,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Universal online file converter supporting 200+ audio, video, document, and image formats. (Channel me kul 2 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: Universal online file converter supporting 200+ audio, video, document, and image formats. (Channel me kul 2 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E3" s="4" t="n">
@@ -611,25 +611,25 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Jobscan</t>
+          <t>Gamma App</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>https://jobscan.co</t>
+          <t>https://gamma.app</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: AI resume scanner that compares your CV against job descriptions to pass ATS filters.</t>
+          <t>Is website se ye sab kar sakte hain: AI-powered presentation, document, and webpage builder that generates styled interactive slide decks from prompts in seconds. (Channel me kul 17 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E5" s="4" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Analyze your resume (https://www.youtube.com/shorts/rmPbzUVbaNE)</t>
+          <t>17 videos (Primary: https://www.youtube.com/shorts/2XNusROtCQQ)</t>
         </is>
       </c>
     </row>
@@ -641,17 +641,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>MuscleWiki</t>
+          <t>GitMind</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>https://musclewiki.com</t>
+          <t>https://gitmind.com</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Interactive visual body map where you click any muscle to get exercise guides and workout plans. (Channel me kul 9 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: Collaborative AI-powered mind mapping and flowchart tool to brainstorm, study, and visually outline complex topics. (Channel me kul 9 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
@@ -659,7 +659,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>9 videos (Primary: https://www.youtube.com/shorts/W-XxRv7qSBw)</t>
+          <t>9 videos (Primary: https://www.youtube.com/shorts/F1UE5hobqLc)</t>
         </is>
       </c>
     </row>
@@ -671,17 +671,17 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Notion</t>
+          <t>Jobscan</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>https://notion.so</t>
+          <t>https://jobscan.co</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: All-in-one workspace for student notes, syllabi, assignment trackers, and wikis.</t>
+          <t>Is website se ye kar sakte hain: AI resume scanner that compares your CV against job descriptions to pass ATS filters.</t>
         </is>
       </c>
       <c r="E7" s="4" t="n">
@@ -689,7 +689,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Organize your study for you (https://www.youtube.com/shorts/jafo7vXs65w)</t>
+          <t>Analyze your resume (https://www.youtube.com/shorts/rmPbzUVbaNE)</t>
         </is>
       </c>
     </row>
@@ -701,25 +701,25 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Omni Calculator</t>
+          <t>MuscleWiki</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>https://omnicalculator.com</t>
+          <t>https://musclewiki.com</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Over 3,000+ smart calculators covering physics, finance, construction, math, and everyday math.</t>
+          <t>Is website se ye sab kar sakte hain: Interactive visual body map where you click any muscle to get exercise guides and workout plans. (Channel me kul 9 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Find all kinds of engineering calculators (https://www.youtube.com/shorts/4CcWAhEj1ME)</t>
+          <t>9 videos (Primary: https://www.youtube.com/shorts/W-XxRv7qSBw)</t>
         </is>
       </c>
     </row>
@@ -731,17 +731,17 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Printify</t>
+          <t>Notion</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>https://printify.com</t>
+          <t>https://notion.so</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Print-on-demand platform for custom merchandise and global e-commerce.</t>
+          <t>Is website se ye sab kar sakte hain: All-in-one connected workspace for student notes, syllabi, assignment trackers, and wikis.</t>
         </is>
       </c>
       <c r="E9" s="4" t="n">
@@ -749,7 +749,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Custom products in minutes (https://www.youtube.com/shorts/v5pfL2wyKEM)</t>
+          <t>Organize your study for you (https://www.youtube.com/shorts/jafo7vXs65w)</t>
         </is>
       </c>
     </row>
@@ -761,25 +761,25 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Reactive Resume</t>
+          <t>Omni Calculator</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>https://rxresu.me</t>
+          <t>https://omnicalculator.com</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Free, open-source, privacy-focused resume builder with customizable layouts and PDF export. (Channel me kul 3 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Over 3,000+ smart calculators covering physics, finance, construction, math, and everyday math.</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>3 videos (Primary: https://www.youtube.com/shorts/To7wD_9SNeI)</t>
+          <t>Find all kinds of engineering calculators (https://www.youtube.com/shorts/4CcWAhEj1ME)</t>
         </is>
       </c>
     </row>
@@ -791,25 +791,25 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Scribe</t>
+          <t>Printify</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>https://scribehow.com</t>
+          <t>https://printify.com</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Automatically turns any digital process into a visual step-by-step guide with screenshots. (Channel me kul 10 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Print-on-demand platform for custom merchandise and global e-commerce.</t>
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>10 videos (Primary: https://www.youtube.com/shorts/9bJHrK94B3w)</t>
+          <t>Custom products in minutes (https://www.youtube.com/shorts/v5pfL2wyKEM)</t>
         </is>
       </c>
     </row>
@@ -821,25 +821,25 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Socialsonic</t>
+          <t>Reactive Resume</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>https://socialsonic.com</t>
+          <t>https://rxresu.me</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: AI social media content creation suite and viral analytics tool.</t>
+          <t>Is website se ye kar sakte hain: Free, open-source, privacy-focused resume builder with customizable layouts and PDF export. (Channel me kul 3 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Create a professional post for LinkedIn in seconds (https://www.youtube.com/shorts/_JQhePLqVxE)</t>
+          <t>3 videos (Primary: https://www.youtube.com/shorts/To7wD_9SNeI)</t>
         </is>
       </c>
     </row>
@@ -851,25 +851,25 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>SuperCook</t>
+          <t>Scribe</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>https://supercook.com</t>
+          <t>https://scribehow.com</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Zero-waste recipe search engine that matches recipes to ingredients you already have at home. (Channel me kul 2 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: Automatically turns any digital workflow into a visual step-by-step guide with screenshots. (Channel me kul 10 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>2 videos (Primary: https://www.youtube.com/shorts/_dpSYyavN_E)</t>
+          <t>10 videos (Primary: https://www.youtube.com/shorts/9bJHrK94B3w)</t>
         </is>
       </c>
     </row>
@@ -881,25 +881,25 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Top 10 powerful websites you s</t>
+          <t>Socialsonic</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>https://tinywow.com</t>
+          <t>https://socialsonic.com</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: Online productivity utilities: Top 10 Powerful Websites You Should Know • Over 200+ free online utility tools for PDF editing, file conversions, and image tools. • Online productivity utilities: Play tons of games • Online productivity utilities: Racing game (Channel me kul 216 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: AI social media content creation suite and viral analytics tool.</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>216</v>
+        <v>1</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>216 videos (Primary: https://www.youtube.com/watch?v=CTizV2M5H6w)</t>
+          <t>Create a professional post for LinkedIn in seconds (https://www.youtube.com/shorts/_JQhePLqVxE)</t>
         </is>
       </c>
     </row>
@@ -911,25 +911,25 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>TypeRacer</t>
+          <t>SuperCook</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>https://play.typeracer.com</t>
+          <t>https://supercook.com</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Multiplayer online typing competition game to test and improve words-per-minute speed. (Channel me kul 17 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: Zero-waste recipe search engine that matches recipes to ingredients you already have at home. (Channel me kul 2 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>17 videos (Primary: https://www.youtube.com/shorts/zPjf9KyHXB4)</t>
+          <t>2 videos (Primary: https://www.youtube.com/shorts/_dpSYyavN_E)</t>
         </is>
       </c>
     </row>
@@ -941,25 +941,25 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Versus</t>
+          <t>TinyWow</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>https://versus.com</t>
+          <t>https://tinywow.com</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Data-driven comparison platform comparing phones, hardware, cities, and software. (Channel me kul 2 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: 200+ free online utility tools: PDF editing/converting/merging, image background removal, file compression, video tools, and AI writing. (Channel me kul 172 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>2</v>
+        <v>172</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2 videos (Primary: https://www.youtube.com/shorts/QDzXMPeVuY0)</t>
+          <t>172 videos (Primary: https://www.youtube.com/watch?v=CTizV2M5H6w)</t>
         </is>
       </c>
     </row>
@@ -971,47 +971,47 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Worksheet Genius</t>
+          <t>TypeRacer</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>https://worksheetgenius.com</t>
+          <t>https://play.typeracer.com</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Free customizable worksheet generator for math problems, vocabulary, and puzzles. (Channel me kul 8 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Multiplayer online typing competition game to test and improve words-per-minute speed. (Channel me kul 17 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>8 videos (Primary: https://www.youtube.com/shorts/0ezJxIveYh4)</t>
+          <t>17 videos (Primary: https://www.youtube.com/shorts/zPjf9KyHXB4)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>🎨 Design, 3D &amp; Graphics</t>
+          <t>⚡ Productivity &amp; Document Tools</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>3DTuning</t>
+          <t>Versus</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>https://3dtuning.com</t>
+          <t>https://versus.com</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Photorealistic 3D car configurator with thousands of car models, body kits, and wheels. (Channel me kul 2 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Data-driven comparison platform comparing phones, hardware, cities, and software. (Channel me kul 2 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
@@ -1019,37 +1019,37 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2 videos (Primary: https://www.youtube.com/shorts/fiaBqxFdlcg)</t>
+          <t>2 videos (Primary: https://www.youtube.com/shorts/QDzXMPeVuY0)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>🎨 Design, 3D &amp; Graphics</t>
+          <t>⚡ Productivity &amp; Document Tools</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Animated Drawings by Meta</t>
+          <t>Worksheet Genius</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>https://sketch.metademolab.com</t>
+          <t>https://worksheetgenius.com</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Animate children's sketches and hand-drawn character drawings into walking, running, and jumping 2D animations. (Channel me kul 3 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Free customizable worksheet generator for math problems, vocabulary, and puzzles. (Channel me kul 8 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>3 videos (Primary: https://www.youtube.com/shorts/VD91M_Qwpi0)</t>
+          <t>8 videos (Primary: https://www.youtube.com/shorts/0ezJxIveYh4)</t>
         </is>
       </c>
     </row>
@@ -1061,25 +1061,25 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Boords</t>
+          <t>3DTuning</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>https://boords.com</t>
+          <t>https://3dtuning.com</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Modern online storyboard creator with AI image generation and script collaboration. (Channel me kul 5 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Photorealistic 3D car configurator with thousands of car models, body kits, and wheels. (Channel me kul 2 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>5 videos (Primary: https://www.youtube.com/shorts/gYWxNAEh2qY)</t>
+          <t>2 videos (Primary: https://www.youtube.com/shorts/fiaBqxFdlcg)</t>
         </is>
       </c>
     </row>
@@ -1091,25 +1091,25 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Freepik Pikaso</t>
+          <t>Animated Drawings by Meta</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>https://freepik.com/pikaso</t>
+          <t>https://sketch.metademolab.com</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Real-time sketch-to-image AI canvas and creative stock assets.</t>
+          <t>Is website se ye kar sakte hain: Animate children's sketches and hand-drawn character drawings into walking, running, and jumping 2D animations. (Channel me kul 3 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E21" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Freepik retouch image (https://www.youtube.com/shorts/QBHAtZNAPEs)</t>
+          <t>3 videos (Primary: https://www.youtube.com/shorts/VD91M_Qwpi0)</t>
         </is>
       </c>
     </row>
@@ -1121,25 +1121,25 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Hero Patterns</t>
+          <t>Boords</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>https://heropatterns.com</t>
+          <t>https://boords.com</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Free collection of repeatable, customizable SVG background patterns for digital design. (Channel me kul 7 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Modern online storyboard creator with AI image generation and script collaboration. (Channel me kul 5 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>7 videos (Primary: https://www.youtube.com/shorts/RZWVLA2x3cE)</t>
+          <t>5 videos (Primary: https://www.youtube.com/shorts/gYWxNAEh2qY)</t>
         </is>
       </c>
     </row>
@@ -1151,17 +1151,17 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Kittl</t>
+          <t>Freepik Pikaso</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>https://kittl.com</t>
+          <t>https://freepik.com/pikaso</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Advanced graphic design platform with AI vector generation and typography.</t>
+          <t>Is website se ye kar sakte hain: Real-time sketch-to-image AI canvas and creative stock assets.</t>
         </is>
       </c>
       <c r="E23" s="4" t="n">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Design logo in seconds (https://www.youtube.com/shorts/P_vtYleN0Oo)</t>
+          <t>Freepik retouch image (https://www.youtube.com/shorts/QBHAtZNAPEs)</t>
         </is>
       </c>
     </row>
@@ -1181,25 +1181,25 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Looka AI</t>
+          <t>Hero Patterns</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>https://looka.com</t>
+          <t>https://heropatterns.com</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: AI-powered logo designer and brand identity generator with complete marketing packages. (Channel me kul 3 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Free collection of repeatable, customizable SVG background patterns for digital design. (Channel me kul 7 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>3 videos (Primary: https://www.youtube.com/shorts/NAJxj01JmhA)</t>
+          <t>7 videos (Primary: https://www.youtube.com/shorts/RZWVLA2x3cE)</t>
         </is>
       </c>
     </row>
@@ -1211,25 +1211,25 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>LottieFiles</t>
+          <t>Kittl</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>https://lottiefiles.com</t>
+          <t>https://kittl.com</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Lightweight, scalable interactive vector Lottie animations for websites and mobile applications. (Channel me kul 2 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Advanced graphic design platform with AI vector generation and typography.</t>
         </is>
       </c>
       <c r="E25" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>2 videos (Primary: https://www.youtube.com/shorts/TGYYO_v9yvY)</t>
+          <t>Design logo in seconds (https://www.youtube.com/shorts/P_vtYleN0Oo)</t>
         </is>
       </c>
     </row>
@@ -1241,25 +1241,25 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>MockupBro</t>
+          <t>Looka AI</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>https://mockupbro.com</t>
+          <t>https://looka.com</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Free online device and product mockup generator with high-resolution instant downloads. (Channel me kul 10 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: AI-powered logo designer and brand identity generator with complete marketing packages. (Channel me kul 3 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>10 videos (Primary: https://www.youtube.com/shorts/JgDOJ10ogsA)</t>
+          <t>3 videos (Primary: https://www.youtube.com/shorts/NAJxj01JmhA)</t>
         </is>
       </c>
     </row>
@@ -1271,25 +1271,25 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Open Peeps</t>
+          <t>LottieFiles</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>https://openpeeps.com</t>
+          <t>https://lottiefiles.com</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Hand-drawn illustration library with customizable facial expressions, poses, and clothing.</t>
+          <t>Is website se ye kar sakte hain: Lightweight, scalable interactive vector Lottie animations for websites and mobile applications. (Channel me kul 2 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Ready to download peeps (https://www.youtube.com/shorts/0XkV6fq0YYo)</t>
+          <t>2 videos (Primary: https://www.youtube.com/shorts/TGYYO_v9yvY)</t>
         </is>
       </c>
     </row>
@@ -1301,25 +1301,25 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Papercurves</t>
+          <t>MockupBro</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>https://papercurves.com</t>
+          <t>https://mockupbro.com</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Interactive 3D paper fold and flip animation generator for creative web interfaces. (Channel me kul 3 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Free online device and product mockup generator with high-resolution instant downloads. (Channel me kul 10 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>3 videos (Primary: https://www.youtube.com/shorts/FDQ3Gr26tm0)</t>
+          <t>10 videos (Primary: https://www.youtube.com/shorts/JgDOJ10ogsA)</t>
         </is>
       </c>
     </row>
@@ -1331,17 +1331,17 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Photopea</t>
+          <t>Open Peeps</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>https://photopea.com</t>
+          <t>https://openpeeps.com</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Advanced browser-based raster and vector photo editor supporting PSD, AI, and RAW files.</t>
+          <t>Is website se ye kar sakte hain: Hand-drawn illustration library with customizable facial expressions, poses, and clothing.</t>
         </is>
       </c>
       <c r="E29" s="4" t="n">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Free AI Photo Editor (https://www.youtube.com/shorts/1sTJf_lQ1lE)</t>
+          <t>Ready to download peeps (https://www.youtube.com/shorts/0XkV6fq0YYo)</t>
         </is>
       </c>
     </row>
@@ -1361,25 +1361,25 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Planner 5D</t>
+          <t>Papercurves</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>https://planner5d.com</t>
+          <t>https://papercurves.com</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Create 2D/3D home floor plans, room layouts, and realistic photorealistic renderings. (Channel me kul 12 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Interactive 3D paper fold and flip animation generator for creative web interfaces. (Channel me kul 3 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>12 videos (Primary: https://www.youtube.com/shorts/79-SKVWfCu8)</t>
+          <t>3 videos (Primary: https://www.youtube.com/shorts/FDQ3Gr26tm0)</t>
         </is>
       </c>
     </row>
@@ -1391,17 +1391,17 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>PosterMyWall</t>
+          <t>Photopea</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>https://postermywall.com</t>
+          <t>https://photopea.com</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Create promotional event posters, social media graphics, and flyer templates in seconds.</t>
+          <t>Is website se ye sab kar sakte hain: Advanced browser-based raster and vector photo editor supporting PSD, AI, and RAW files without installation.</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Create stunning posters in seconds (https://www.youtube.com/shorts/BmdieiOXfyM)</t>
+          <t>Free AI Photo Editor (https://www.youtube.com/shorts/1sTJf_lQ1lE)</t>
         </is>
       </c>
     </row>
@@ -1421,25 +1421,25 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Renderforest 3D Logo</t>
+          <t>Planner 5D</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>https://renderforest.com</t>
+          <t>https://planner5d.com</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Transform 2D brand logos into animated 3D video openers and intros in minutes. (Channel me kul 3 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Create 2D/3D home floor plans, room layouts, and realistic photorealistic renderings. (Channel me kul 12 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>3 videos (Primary: https://www.youtube.com/shorts/w8oMMUMQPTY)</t>
+          <t>12 videos (Primary: https://www.youtube.com/shorts/79-SKVWfCu8)</t>
         </is>
       </c>
     </row>
@@ -1451,17 +1451,17 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Shapefest</t>
+          <t>PosterMyWall</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>https://shapefest.com</t>
+          <t>https://postermywall.com</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Massive library of 30,000+ free high-resolution 3D clay, plastic, and metal icons and hand gestures.</t>
+          <t>Is website se ye kar sakte hain: Create promotional event posters, social media graphics, and flyer templates in seconds.</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Find almost any 3D PNG icons (https://www.youtube.com/shorts/57h13k9Ym4Q)</t>
+          <t>Create stunning posters in seconds (https://www.youtube.com/shorts/BmdieiOXfyM)</t>
         </is>
       </c>
     </row>
@@ -1481,25 +1481,25 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Threed.io</t>
+          <t>Renderforest 3D Logo</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>https://threed.io</t>
+          <t>https://renderforest.com</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Generate custom 3D device and packaging mockups directly in your web browser with real-time controls.</t>
+          <t>Is website se ye kar sakte hain: Transform 2D brand logos into animated 3D video openers and intros in minutes. (Channel me kul 3 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Generate a complete product design (https://www.youtube.com/shorts/OzmI9iXTY5g)</t>
+          <t>3 videos (Primary: https://www.youtube.com/shorts/w8oMMUMQPTY)</t>
         </is>
       </c>
     </row>
@@ -1511,25 +1511,25 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Toools.design</t>
+          <t>Shapefest</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>https://toools.design</t>
+          <t>https://shapefest.com</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: Curated directory of 1,000+ modern design tools, mockups, typography, and resources. • Creative design utility: Instantly creates a 3D map • Creative design utility: Logo animation • Creative design utility: Find almost any cursor style (Channel me kul 128 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Massive library of 30,000+ free high-resolution 3D clay, plastic, and metal icons and hand gestures.</t>
         </is>
       </c>
       <c r="E35" s="4" t="n">
-        <v>128</v>
+        <v>1</v>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>128 videos (Primary: https://www.youtube.com/shorts/jJaVCb0qy60)</t>
+          <t>Find almost any 3D PNG icons (https://www.youtube.com/shorts/57h13k9Ym4Q)</t>
         </is>
       </c>
     </row>
@@ -1541,25 +1541,25 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Uiverse.io</t>
+          <t>Threed.io</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>https://uiverse.io</t>
+          <t>https://threed.io</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: World's largest open-source library of community-made CSS and Tailwind animated UI elements. (Channel me kul 10 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Generate custom 3D device and packaging mockups directly in your web browser with real-time controls.</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>10 videos (Primary: https://www.youtube.com/shorts/tdyo7l5D9O8)</t>
+          <t>Generate a complete product design (https://www.youtube.com/shorts/OzmI9iXTY5g)</t>
         </is>
       </c>
     </row>
@@ -1571,25 +1571,25 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Uizard</t>
+          <t>Toools.design</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>https://uizard.io</t>
+          <t>https://toools.design</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: AI UI/UX design tool that transforms hand-drawn wireframes and screenshots into editable digital designs.</t>
+          <t>Is website se ye sab kar sakte hain: Curated repository of 1,000+ modern design tools, mockups, typography, illustration packs, and UI kits. (Channel me kul 166 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E37" s="4" t="n">
-        <v>1</v>
+        <v>166</v>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Create a professional UI design just by text (https://www.youtube.com/shorts/EKSrht47q4Y)</t>
+          <t>166 videos (Primary: https://www.youtube.com/shorts/jJaVCb0qy60)</t>
         </is>
       </c>
     </row>
@@ -1601,25 +1601,25 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Vectorizer.AI</t>
+          <t>Uiverse.io</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>https://vectorizer.ai</t>
+          <t>https://uiverse.io</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Convert raster blurry JPEG/PNG images into crisp, scalable SVG vectors using deep learning.</t>
+          <t>Is website se ye sab kar sakte hain: World's largest open-source library of community-made CSS and Tailwind animated UI elements, buttons, and switches. (Channel me kul 10 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Turn blurry image into vector (https://www.youtube.com/shorts/8XhlbCYCu1k)</t>
+          <t>10 videos (Primary: https://www.youtube.com/shorts/tdyo7l5D9O8)</t>
         </is>
       </c>
     </row>
@@ -1631,17 +1631,17 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Weavesilk</t>
+          <t>Uizard</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>https://weavesilk.com</t>
+          <t>https://uizard.io</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Interactive generative art canvas with glowing symmetry and cloth-like interactive flow.</t>
+          <t>Is website se ye kar sakte hain: AI UI/UX design tool that transforms hand-drawn wireframes and screenshots into editable digital designs.</t>
         </is>
       </c>
       <c r="E39" s="4" t="n">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Create holographic and cloth like effects in your browser (https://www.youtube.com/shorts/aMjQA1YA3As)</t>
+          <t>Create a professional UI design just by text (https://www.youtube.com/shorts/EKSrht47q4Y)</t>
         </is>
       </c>
     </row>
@@ -1661,17 +1661,17 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Wondershare Filmora</t>
+          <t>Vectorizer.AI</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>https://filmora.wondershare.com</t>
+          <t>https://vectorizer.ai</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Video editing software with AI smart cutout, audio ducking, and effects.</t>
+          <t>Is website se ye kar sakte hain: Convert raster blurry JPEG/PNG images into crisp, scalable SVG vectors using deep learning.</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
@@ -1679,59 +1679,59 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Turn your long videos into shorts with Filmora V14 (https://www.youtube.com/shorts/GfqGDPv6N48)</t>
+          <t>Turn blurry image into vector (https://www.youtube.com/shorts/8XhlbCYCu1k)</t>
         </is>
       </c>
     </row>
     <row r="41" ht="24" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>🎮 Gaming &amp; Fun Web Experiments</t>
+          <t>🎨 Design, 3D &amp; Graphics</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Azgaar's Fantasy Map Generator</t>
+          <t>Weavesilk</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>https://azgaar.github.io/Fantasy-Map-Generator/</t>
+          <t>https://weavesilk.com</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Procedural world map generator creating medieval fantasy realms with rivers, cities, and biomes. (Channel me kul 3 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Interactive generative art canvas with glowing symmetry and cloth-like interactive flow.</t>
         </is>
       </c>
       <c r="E41" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>3 videos (Primary: https://www.youtube.com/shorts/nKI-qz6pmUM)</t>
+          <t>Create holographic and cloth like effects in your browser (https://www.youtube.com/shorts/aMjQA1YA3As)</t>
         </is>
       </c>
     </row>
     <row r="42" ht="24" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>🎮 Gaming &amp; Fun Web Experiments</t>
+          <t>🎨 Design, 3D &amp; Graphics</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Before I Play</t>
+          <t>Wondershare Filmora</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>https://beforeiplay.com</t>
+          <t>https://filmora.wondershare.com</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Crowdsourced spoiler-free tips, essential advice, and misses before starting any video game.</t>
+          <t>Is website se ye kar sakte hain: Video editing software with AI smart cutout, audio ducking, and effects.</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Before I Play (https://www.youtube.com/shorts/yCdcyeNjvho)</t>
+          <t>Turn your long videos into shorts with Filmora V14 (https://www.youtube.com/shorts/GfqGDPv6N48)</t>
         </is>
       </c>
     </row>
@@ -1751,25 +1751,25 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Funkypot 3D Snooker</t>
+          <t>Azgaar's Fantasy Map Generator</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>https://funkypot.com</t>
+          <t>https://azgaar.github.io/Fantasy-Map-Generator/</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Realistic 3D browser snooker and billiards physics simulation game.</t>
+          <t>Is website se ye kar sakte hain: Procedural world map generator creating medieval fantasy realms with rivers, cities, and biomes. (Channel me kul 3 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E43" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>3D snooker (https://www.youtube.com/shorts/Q2oDYTP1hFM)</t>
+          <t>3 videos (Primary: https://www.youtube.com/shorts/nKI-qz6pmUM)</t>
         </is>
       </c>
     </row>
@@ -1781,17 +1781,17 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Kick Ass Web Destroyer</t>
+          <t>Before I Play</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>https://kickassapp.com</t>
+          <t>https://beforeiplay.com</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Asteroids-style browser game bookmarklet that blasts and deletes HTML elements on any webpage.</t>
+          <t>Is website se ye kar sakte hain: Crowdsourced spoiler-free tips, essential advice, and misses before starting any video game.</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>A game where you break apart website design elements (https://www.youtube.com/shorts/1cQpi9dki1s)</t>
+          <t>Before I Play (https://www.youtube.com/shorts/yCdcyeNjvho)</t>
         </is>
       </c>
     </row>
@@ -1811,17 +1811,17 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Line Rider</t>
+          <t>Funkypot 3D Snooker</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>https://linerider.com</t>
+          <t>https://funkypot.com</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Physics drawing sandbox game where you create slopes and tracks for a sledder.</t>
+          <t>Is website se ye kar sakte hain: Realistic 3D browser snooker and billiards physics simulation game.</t>
         </is>
       </c>
       <c r="E45" s="4" t="n">
@@ -1829,7 +1829,7 @@
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Draw your racetrack (https://www.youtube.com/shorts/UZk2XUiigqI)</t>
+          <t>3D snooker (https://www.youtube.com/shorts/Q2oDYTP1hFM)</t>
         </is>
       </c>
     </row>
@@ -1841,17 +1841,17 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Neave Interactive</t>
+          <t>Kick Ass Web Destroyer</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>https://neave.com</t>
+          <t>https://kickassapp.com</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Collection of minimalist retro browser games and fun interactive creative experiments.</t>
+          <t>Is website se ye kar sakte hain: Asteroids-style browser game bookmarklet that blasts and deletes HTML elements on any webpage.</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Stack your ice cream (https://www.youtube.com/shorts/A-kr7nsdRmY)</t>
+          <t>A game where you break apart website design elements (https://www.youtube.com/shorts/1cQpi9dki1s)</t>
         </is>
       </c>
     </row>
@@ -1871,25 +1871,25 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Slow Roads</t>
+          <t>Line Rider</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>https://slowroads.io</t>
+          <t>https://linerider.com</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Infinite, relaxing procedural 3D driving simulator running smoothly in the browser. (Channel me kul 2 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Physics drawing sandbox game where you create slopes and tracks for a sledder.</t>
         </is>
       </c>
       <c r="E47" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>2 videos (Primary: https://www.youtube.com/shorts/m1DRC_Iufvo)</t>
+          <t>Draw your racetrack (https://www.youtube.com/shorts/UZk2XUiigqI)</t>
         </is>
       </c>
     </row>
@@ -1901,17 +1901,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Smashboards</t>
+          <t>Neave Interactive</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>https://smashboards.com</t>
+          <t>https://neave.com</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: The world premier Super Smash Bros community, retro editions, and browser tournaments.</t>
+          <t>Is website se ye kar sakte hain: Collection of minimalist retro browser games and fun interactive creative experiments.</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
@@ -1919,29 +1919,29 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Super Smash Brothers (https://www.youtube.com/shorts/8zoODgWzxV4)</t>
+          <t>Stack your ice cream (https://www.youtube.com/shorts/A-kr7nsdRmY)</t>
         </is>
       </c>
     </row>
     <row r="49" ht="24" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>🎵 Audio, Voice &amp; Music</t>
+          <t>🎮 Gaming &amp; Fun Web Experiments</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Chordify</t>
+          <t>Slow Roads</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>https://chordify.net</t>
+          <t>https://slowroads.io</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Extract chords and learn to play any song on guitar, piano, or ukulele in real time. (Channel me kul 2 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Infinite, relaxing procedural 3D driving simulator running smoothly in the browser. (Channel me kul 2 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E49" s="4" t="n">
@@ -1949,29 +1949,29 @@
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>2 videos (Primary: https://www.youtube.com/shorts/stI1Jjfm4hA)</t>
+          <t>2 videos (Primary: https://www.youtube.com/shorts/m1DRC_Iufvo)</t>
         </is>
       </c>
     </row>
     <row r="50" ht="24" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>🎵 Audio, Voice &amp; Music</t>
+          <t>🎮 Gaming &amp; Fun Web Experiments</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Podcastle</t>
+          <t>Smashboards</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>https://podcastle.ai</t>
+          <t>https://smashboards.com</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Studio-quality audio recording, noise removal, and AI voice editing suite.</t>
+          <t>Is website se ye kar sakte hain: The world premier Super Smash Bros community, retro editions, and browser tournaments.</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Make you sound professional (https://www.youtube.com/shorts/SpXtgZ40Ibk)</t>
+          <t>Super Smash Brothers (https://www.youtube.com/shorts/8zoODgWzxV4)</t>
         </is>
       </c>
     </row>
@@ -1991,17 +1991,17 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Radio Garden</t>
+          <t>Chordify</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>https://radio.garden</t>
+          <t>https://chordify.net</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Explore and listen to thousands of live radio stations worldwide on a 3D digital globe. (Channel me kul 2 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Extract chords and learn to play any song on guitar, piano, or ukulele in real time. (Channel me kul 2 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E51" s="4" t="n">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>2 videos (Primary: https://www.youtube.com/shorts/Xhw_CpPJdcI)</t>
+          <t>2 videos (Primary: https://www.youtube.com/shorts/stI1Jjfm4hA)</t>
         </is>
       </c>
     </row>
@@ -2021,115 +2021,115 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Vocal Remover</t>
+          <t>Podcastle</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>https://vocalremover.org</t>
+          <t>https://podcastle.ai</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: AI-powered online audio tool that isolates vocals and instrumental tracks for free. • Audio manipulation: Play your favorite song • Audio manipulation: Remove echo and background noise • Audio manipulation: Learn music theory through interactive simulations (Channel me kul 20 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Studio-quality audio recording, noise removal, and AI voice editing suite.</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>20 videos (Primary: https://www.youtube.com/shorts/1lOPX_U4ljQ)</t>
+          <t>Make you sound professional (https://www.youtube.com/shorts/SpXtgZ40Ibk)</t>
         </is>
       </c>
     </row>
     <row r="53" ht="24" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>💻 Coding &amp; Web Development</t>
+          <t>🎵 Audio, Voice &amp; Music</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Falstad Circuit Simulator</t>
+          <t>Radio Garden</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>https://falstad.com/circuit</t>
+          <t>https://radio.garden</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Interactive browser electronic circuit simulator visualizing currents, AC/DC, and logic gates. (Channel me kul 7 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Explore and listen to thousands of live radio stations worldwide on a 3D digital globe. (Channel me kul 2 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E53" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>7 videos (Primary: https://www.youtube.com/shorts/Z6NuZRM899g)</t>
+          <t>2 videos (Primary: https://www.youtube.com/shorts/Xhw_CpPJdcI)</t>
         </is>
       </c>
     </row>
     <row r="54" ht="24" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>💻 Coding &amp; Web Development</t>
+          <t>🎵 Audio, Voice &amp; Music</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Framer</t>
+          <t>Udio</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>https://framer.com</t>
+          <t>https://udio.com</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: AI-powered no-code website builder that creates responsive production-ready sites. • No-code interactive website builder with instant production deployment. (Channel me kul 11 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: High-fidelity AI music generation engine capable of generating full tracks from prompts. (Channel me kul 5 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>11 videos (Primary: https://www.youtube.com/shorts/BiYVT88VRn8)</t>
+          <t>5 videos (Primary: https://www.youtube.com/shorts/_E4tOZooHgk)</t>
         </is>
       </c>
     </row>
     <row r="55" ht="24" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>💻 Coding &amp; Web Development</t>
+          <t>🎵 Audio, Voice &amp; Music</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Replit</t>
+          <t>Vocal Remover</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>https://replit.com</t>
+          <t>https://vocalremover.org</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: Cloud software creation and instant AI web app hosting platform. • Development &amp; code features: Creative QR code generator • Development &amp; code features: Learn coding like a game • Development &amp; code features: Build almost anything (Channel me kul 72 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: AI-powered online audio tool that isolates vocals and instrumental tracks for free. (Channel me kul 18 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E55" s="4" t="n">
-        <v>72</v>
+        <v>18</v>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>72 videos (Primary: https://www.youtube.com/shorts/7GSm4UKSY94)</t>
+          <t>18 videos (Primary: https://www.youtube.com/shorts/1lOPX_U4ljQ)</t>
         </is>
       </c>
     </row>
@@ -2141,25 +2141,25 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Runable AI</t>
+          <t>Falstad Circuit Simulator</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>https://runable.ai</t>
+          <t>https://falstad.com/circuit</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Natural language prompt-to-app generator that codes complete full-stack web applications. (Channel me kul 2 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Interactive browser electronic circuit simulator visualizing currents, AC/DC, and logic gates. (Channel me kul 7 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2 videos (Primary: https://www.youtube.com/shorts/Cuql4B-m1VI)</t>
+          <t>7 videos (Primary: https://www.youtube.com/shorts/Z6NuZRM899g)</t>
         </is>
       </c>
     </row>
@@ -2171,115 +2171,115 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Wegic AI</t>
+          <t>Framer</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>https://wegic.ai</t>
+          <t>https://framer.com</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Conversational AI web designer that crafts responsive websites through chat.</t>
+          <t>Is website se ye sab kar sakte hain: AI-powered no-code website builder that creates responsive production-ready sites. • No-code interactive website builder with instant production deployment. (Channel me kul 11 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E57" s="4" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>Create a website with zero coding (https://www.youtube.com/shorts/gu8AiSj29_0)</t>
+          <t>11 videos (Primary: https://www.youtube.com/shorts/BiYVT88VRn8)</t>
         </is>
       </c>
     </row>
     <row r="58" ht="24" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>📚 Learning, Study &amp; Research</t>
+          <t>💻 Coding &amp; Web Development</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Animated Engines</t>
+          <t>Replit</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>https://animatedengines.com</t>
+          <t>https://replit.com</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Detailed animated mechanical breakdowns showing how combustion and jet engines work. (Channel me kul 3 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: Collaborative browser-based IDE, AI code generation, and instant cloud application deployment workspace. (Channel me kul 52 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>3</v>
+        <v>52</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>3 videos (Primary: https://www.youtube.com/shorts/5iWCRa5LhGo)</t>
+          <t>52 videos (Primary: https://www.youtube.com/shorts/7GSm4UKSY94)</t>
         </is>
       </c>
     </row>
     <row r="59" ht="24" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>📚 Learning, Study &amp; Research</t>
+          <t>💻 Coding &amp; Web Development</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Anything</t>
+          <t>Runable AI</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>https://quillbot.com</t>
+          <t>https://runable.ai</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: Study &amp; academic utility: Learn almost anything • Study &amp; academic utility: Find almost any live wallpapers • Study &amp; academic utility: Generate Duolingo style study plan • Study &amp; academic utility: Simulate almost any chemistry experiment (Channel me kul 62 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Natural language prompt-to-app generator that codes complete full-stack web applications. (Channel me kul 2 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E59" s="4" t="n">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>62 videos (Primary: https://www.youtube.com/shorts/9l2xxSl7MYI)</t>
+          <t>2 videos (Primary: https://www.youtube.com/shorts/Cuql4B-m1VI)</t>
         </is>
       </c>
     </row>
     <row r="60" ht="24" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>📚 Learning, Study &amp; Research</t>
+          <t>💻 Coding &amp; Web Development</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Auto-Brochures</t>
+          <t>Wegic AI</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>https://auto-brochures.com</t>
+          <t>https://wegic.ai</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Free archive of classic and modern automotive factory brochures and spec sheets. (Channel me kul 2 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Conversational AI web designer that crafts responsive websites through chat.</t>
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2 videos (Primary: https://www.youtube.com/shorts/AYdHYLZiw6A)</t>
+          <t>Create a website with zero coding (https://www.youtube.com/shorts/gu8AiSj29_0)</t>
         </is>
       </c>
     </row>
@@ -2291,25 +2291,25 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Ba Ba Dum</t>
+          <t>Animated Engines</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>https://babadum.com</t>
+          <t>https://animatedengines.com</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Visual browser game teaching 1,500 core words across 21 global languages. (Channel me kul 2 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Detailed animated mechanical breakdowns showing how combustion and jet engines work. (Channel me kul 3 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E61" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>2 videos (Primary: https://www.youtube.com/shorts/e2sm6TNPbbA)</t>
+          <t>3 videos (Primary: https://www.youtube.com/shorts/5iWCRa5LhGo)</t>
         </is>
       </c>
     </row>
@@ -2321,25 +2321,25 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>BioDigital Human</t>
+          <t>Auto-Brochures</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>https://biodigital.com</t>
+          <t>https://auto-brochures.com</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Interactive 3D model of the human anatomy, diseases, and medical treatments. (Channel me kul 7 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Free archive of classic and modern automotive factory brochures and spec sheets. (Channel me kul 2 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>7 videos (Primary: https://www.youtube.com/shorts/vmjU4OcKfko)</t>
+          <t>2 videos (Primary: https://www.youtube.com/shorts/AYdHYLZiw6A)</t>
         </is>
       </c>
     </row>
@@ -2351,25 +2351,25 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>CameraSim</t>
+          <t>Ba Ba Dum</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>https://camerasim.com</t>
+          <t>https://babadum.com</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Interactive SLR camera simulator teaching aperture, shutter speed, and ISO exposure.</t>
+          <t>Is website se ye kar sakte hain: Visual browser game teaching 1,500 core words across 21 global languages. (Channel me kul 2 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E63" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>See how diffident camera settings work together (https://www.youtube.com/shorts/wXw1GBJau6g)</t>
+          <t>2 videos (Primary: https://www.youtube.com/shorts/e2sm6TNPbbA)</t>
         </is>
       </c>
     </row>
@@ -2381,25 +2381,25 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>How a Car Works</t>
+          <t>BioDigital Human</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>https://howacarworks.com</t>
+          <t>https://biodigital.com</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Comprehensive video guide and interactive technical diagrams of car mechanics. (Channel me kul 3 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: Interactive 3D virtual human anatomy atlas and disease explorer for medical students, healthcare pros, and biology. (Channel me kul 7 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>3 videos (Primary: https://www.youtube.com/shorts/yVMKHnQ_y0w)</t>
+          <t>7 videos (Primary: https://www.youtube.com/shorts/vmjU4OcKfko)</t>
         </is>
       </c>
     </row>
@@ -2411,17 +2411,17 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Mindgrasp AI</t>
+          <t>CameraSim</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>https://mindgrasp.ai</t>
+          <t>https://camerasim.com</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: AI study assistant that summarizes lectures, PDFs, and generates flashcards.</t>
+          <t>Is website se ye kar sakte hain: Interactive SLR camera simulator teaching aperture, shutter speed, and ISO exposure.</t>
         </is>
       </c>
       <c r="E65" s="4" t="n">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>Do research in seconds Ai (https://www.youtube.com/shorts/_OowyGXsN3w)</t>
+          <t>See how diffident camera settings work together (https://www.youtube.com/shorts/wXw1GBJau6g)</t>
         </is>
       </c>
     </row>
@@ -2441,25 +2441,25 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>PhET Interactive Simulations</t>
+          <t>Coursera</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>https://phet.colorado.edu</t>
+          <t>https://coursera.org</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Research-backed interactive science simulations by the University of Colorado Boulder. (Channel me kul 4 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: Global online learning platform offering courses and degrees from top universities like Stanford and Yale. (Channel me kul 3 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E66" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>4 videos (Primary: https://www.youtube.com/shorts/ftmSlliTFRQ)</t>
+          <t>3 videos (Primary: https://www.youtube.com/shorts/swfy1eb_ftU)</t>
         </is>
       </c>
     </row>
@@ -2471,17 +2471,17 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Quickposes</t>
+          <t>Grow with Google</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>https://quickposes.com</t>
+          <t>https://grow.google/certificates/interview-warmup/</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Timed gesture drawing and pose reference generator for digital artists and sketchers.</t>
+          <t>Is website se ye sab kar sakte hain: Google's official certification programs offering free training in AI, data analytics, project management, and IT.</t>
         </is>
       </c>
       <c r="E67" s="4" t="n">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>Perfect for practicing portraits (https://www.youtube.com/shorts/PUu4EZ0h7xg)</t>
+          <t>Interview candidates with AI (https://www.youtube.com/shorts/SYVGhej9N5M)</t>
         </is>
       </c>
     </row>
@@ -2501,47 +2501,47 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Unriddle AI</t>
+          <t>How a Car Works</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>https://unriddle.ai</t>
+          <t>https://howacarworks.com</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: AI research companion to read, understand, and chat with technical documents.</t>
+          <t>Is website se ye kar sakte hain: Comprehensive video guide and interactive technical diagrams of car mechanics. (Channel me kul 3 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Chat with pdf &amp; use ChatGPT for free (https://www.youtube.com/shorts/aZWVNDEZM30)</t>
+          <t>3 videos (Primary: https://www.youtube.com/shorts/yVMKHnQ_y0w)</t>
         </is>
       </c>
     </row>
     <row r="69" ht="24" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>🗺️ Maps, 3D &amp; Exploration</t>
+          <t>📚 Learning, Study &amp; Research</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Ancient Earth Globe</t>
+          <t>Mindgrasp AI</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>https://dinosaurpictures.org/ancient-earth</t>
+          <t>https://mindgrasp.ai</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Interactive 3D visualization of Earth spanning 750 million years of continental drift.</t>
+          <t>Is website se ye kar sakte hain: AI study assistant that summarizes lectures, PDFs, and generates flashcards.</t>
         </is>
       </c>
       <c r="E69" s="4" t="n">
@@ -2549,127 +2549,127 @@
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>Ancient earth (https://www.youtube.com/shorts/0ChxN6YQJc8)</t>
+          <t>Do research in seconds Ai (https://www.youtube.com/shorts/_OowyGXsN3w)</t>
         </is>
       </c>
     </row>
     <row r="70" ht="24" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>🗺️ Maps, 3D &amp; Exploration</t>
+          <t>📚 Learning, Study &amp; Research</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>BlueMap</t>
+          <t>PhET Interactive Simulations</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>https://bluemap.bluecolored.de</t>
+          <t>https://phet.colorado.edu</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Renders 3D interactive, zoomable real-time web maps of Minecraft worlds. (Channel me kul 2 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: Research-backed interactive science and math simulations by University of Colorado Boulder for chemistry and physics. (Channel me kul 4 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E70" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2 videos (Primary: https://www.youtube.com/shorts/Go7LRm88ZX4)</t>
+          <t>4 videos (Primary: https://www.youtube.com/shorts/ftmSlliTFRQ)</t>
         </is>
       </c>
     </row>
     <row r="71" ht="24" customHeight="1">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>🗺️ Maps, 3D &amp; Exploration</t>
+          <t>📚 Learning, Study &amp; Research</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>City-roads by Anvaka</t>
+          <t>Quickposes</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>https://anvaka.github.io/city-roads</t>
+          <t>https://quickposes.com</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Visualizes every single road of any city in the world as minimalist vector art. (Channel me kul 5 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Timed gesture drawing and pose reference generator for digital artists and sketchers.</t>
         </is>
       </c>
       <c r="E71" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>5 videos (Primary: https://www.youtube.com/shorts/ckB1XezyhMI)</t>
+          <t>Perfect for practicing portraits (https://www.youtube.com/shorts/PUu4EZ0h7xg)</t>
         </is>
       </c>
     </row>
     <row r="72" ht="24" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>🗺️ Maps, 3D &amp; Exploration</t>
+          <t>📚 Learning, Study &amp; Research</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>EarthCam</t>
+          <t>QuillBot</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>https://earthcam.com</t>
+          <t>https://quillbot.com</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: Live streaming webcams showcasing famous landmarks, skylines, and world events. • Interactive map &amp; location views: generate an entire fantasy world from scratch • Interactive map &amp; location views: Drive on map • Interactive map &amp; location views: Fly anywhere in the world (Channel me kul 27 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: AI paraphrasing, grammar checking, academic summarization, plagiarism detection, and student thesis writing assistance. (Channel me kul 61 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E72" s="2" t="n">
-        <v>27</v>
+        <v>61</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>27 videos (Primary: https://www.youtube.com/shorts/DpHqeVhCruE)</t>
+          <t>61 videos (Primary: https://www.youtube.com/shorts/9l2xxSl7MYI)</t>
         </is>
       </c>
     </row>
     <row r="73" ht="24" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>🗺️ Maps, 3D &amp; Exploration</t>
+          <t>📚 Learning, Study &amp; Research</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Flightradar24</t>
+          <t>Unriddle AI</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>https://flightradar24.com</t>
+          <t>https://unriddle.ai</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Real-time global aircraft and flight tracker with detailed flight route data. (Channel me kul 2 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: AI research companion to read, understand, and chat with technical documents.</t>
         </is>
       </c>
       <c r="E73" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>2 videos (Primary: https://www.youtube.com/shorts/_0hbWKKJox0)</t>
+          <t>Chat with pdf &amp; use ChatGPT for free (https://www.youtube.com/shorts/aZWVNDEZM30)</t>
         </is>
       </c>
     </row>
@@ -2681,25 +2681,25 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Roadtrippers</t>
+          <t>Ancient Earth Globe</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>https://roadtrippers.com</t>
+          <t>https://dinosaurpictures.org/ancient-earth</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Ultimate road trip route planner finding unique roadside attractions and scenic spots. (Channel me kul 9 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Interactive 3D visualization of Earth spanning 750 million years of continental drift.</t>
         </is>
       </c>
       <c r="E74" s="2" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>9 videos (Primary: https://www.youtube.com/shorts/USpkZlj9ac0)</t>
+          <t>Ancient earth (https://www.youtube.com/shorts/0ChxN6YQJc8)</t>
         </is>
       </c>
     </row>
@@ -2711,25 +2711,25 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>The True Size Of</t>
+          <t>BlueMap</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>https://thetruesize.com</t>
+          <t>https://bluemap.bluecolored.de</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Drag countries across the globe to discover their true scale without map distortion. (Channel me kul 3 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Renders 3D interactive, zoomable real-time web maps of Minecraft worlds. (Channel me kul 2 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E75" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>3 videos (Primary: https://www.youtube.com/shorts/E64YMRaNcZw)</t>
+          <t>2 videos (Primary: https://www.youtube.com/shorts/Go7LRm88ZX4)</t>
         </is>
       </c>
     </row>
@@ -2741,167 +2741,167 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>TouchTerrain</t>
+          <t>City-roads by Anvaka</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>https://touchterrain.geol.iastate.edu</t>
+          <t>https://anvaka.github.io/city-roads</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Converts geographic digital elevation maps into 3D printable STL terrain models.</t>
+          <t>Is website se ye kar sakte hain: Visualizes every single road of any city in the world as minimalist vector art. (Channel me kul 5 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Instantly turn the map into a 3D model (https://www.youtube.com/shorts/IHLXFoKc2d4)</t>
+          <t>5 videos (Primary: https://www.youtube.com/shorts/ckB1XezyhMI)</t>
         </is>
       </c>
     </row>
     <row r="77" ht="24" customHeight="1">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>🛠️ Utilities &amp; Web Tools</t>
+          <t>🗺️ Maps, 3D &amp; Exploration</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Brickit App</t>
+          <t>EarthCam</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>https://brickit.app</t>
+          <t>https://earthcam.com</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: AI app that scans LEGO piles on the floor and gives step-by-step build ideas.</t>
+          <t>Is website se ye sab kar sakte hain: Global network of live streaming webcams providing scenic and landmark views worldwide. (Channel me kul 41 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E77" s="4" t="n">
-        <v>1</v>
+        <v>41</v>
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>Generate tons of ideas based on your bricks (https://www.youtube.com/shorts/G8Akt4gCPYc)</t>
+          <t>41 videos (Primary: https://www.youtube.com/shorts/DpHqeVhCruE)</t>
         </is>
       </c>
     </row>
     <row r="78" ht="24" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>🛠️ Utilities &amp; Web Tools</t>
+          <t>🗺️ Maps, 3D &amp; Exploration</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>iFixit</t>
+          <t>Flightradar24</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>https://ifixit.com</t>
+          <t>https://flightradar24.com</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Free global repair manuals, teardowns, and gadget troubleshooting step-by-step guides. (Channel me kul 17 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Real-time global aircraft and flight tracker with detailed flight route data. (Channel me kul 2 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>17 videos (Primary: https://www.youtube.com/shorts/r0DFTP6V-cY)</t>
+          <t>2 videos (Primary: https://www.youtube.com/shorts/_0hbWKKJox0)</t>
         </is>
       </c>
     </row>
     <row r="79" ht="24" customHeight="1">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>🤖 AI &amp; Machine Learning Tools</t>
+          <t>🗺️ Maps, 3D &amp; Exploration</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Coze AI</t>
+          <t>Roadtrippers</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>https://coze.com</t>
+          <t>https://roadtrippers.com</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: All-in-one AI bot creation platform powered by GPT-4 and advanced plugins for free.</t>
+          <t>Is website se ye kar sakte hain: Ultimate road trip route planner finding unique roadside attractions and scenic spots. (Channel me kul 9 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E79" s="4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>Use ChatGPT for free (https://www.youtube.com/shorts/RgsWlLhZ7V0)</t>
+          <t>9 videos (Primary: https://www.youtube.com/shorts/USpkZlj9ac0)</t>
         </is>
       </c>
     </row>
     <row r="80" ht="24" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>🤖 AI &amp; Machine Learning Tools</t>
+          <t>🗺️ Maps, 3D &amp; Exploration</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Flair.ai</t>
+          <t>The True Size Of</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>https://flair.ai</t>
+          <t>https://thetruesize.com</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: AI product photography studio generating high-end commercial photo shoots in seconds.</t>
+          <t>Is website se ye kar sakte hain: Drag countries across the globe to discover their true scale without map distortion. (Channel me kul 3 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>AI create multiple product images (https://www.youtube.com/shorts/9QpXxmx_HFY)</t>
+          <t>3 videos (Primary: https://www.youtube.com/shorts/E64YMRaNcZw)</t>
         </is>
       </c>
     </row>
     <row r="81" ht="24" customHeight="1">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>🤖 AI &amp; Machine Learning Tools</t>
+          <t>🗺️ Maps, 3D &amp; Exploration</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Gamma App</t>
+          <t>TouchTerrain</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>https://gamma.app</t>
+          <t>https://touchterrain.geol.iastate.edu</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: AI presentation, document, and webpage builder in seconds.</t>
+          <t>Is website se ye kar sakte hain: Converts geographic digital elevation maps into 3D printable STL terrain models.</t>
         </is>
       </c>
       <c r="E81" s="4" t="n">
@@ -2909,67 +2909,67 @@
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>Generate presentation in seconds (https://www.youtube.com/shorts/MIZHHL7K6kY)</t>
+          <t>Instantly turn the map into a 3D model (https://www.youtube.com/shorts/IHLXFoKc2d4)</t>
         </is>
       </c>
     </row>
     <row r="82" ht="24" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>🤖 AI &amp; Machine Learning Tools</t>
+          <t>🛠️ Utilities &amp; Web Tools</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>InVideo AI</t>
+          <t>Brickit App</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>https://invideo.io</t>
+          <t>https://brickit.app</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Full text-to-video AI generator that creates complete edited shorts with voiceovers. (Channel me kul 2 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: AI app that scans LEGO piles on the floor and gives step-by-step build ideas.</t>
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2 videos (Primary: https://www.youtube.com/shorts/f6dw_9E-6ss)</t>
+          <t>Generate tons of ideas based on your bricks (https://www.youtube.com/shorts/G8Akt4gCPYc)</t>
         </is>
       </c>
     </row>
     <row r="83" ht="24" customHeight="1">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>🤖 AI &amp; Machine Learning Tools</t>
+          <t>🛠️ Utilities &amp; Web Tools</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>InstantID</t>
+          <t>iFixit</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>https://github.com/InstantID/InstantID</t>
+          <t>https://ifixit.com</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: State-of-the-art zero-shot identity-preserving image synthesis method.</t>
+          <t>Is website se ye kar sakte hain: Free global repair manuals, teardowns, and gadget troubleshooting step-by-step guides. (Channel me kul 17 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E83" s="4" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>Instant ID (https://www.youtube.com/shorts/VGvqzzW4OZc)</t>
+          <t>17 videos (Primary: https://www.youtube.com/shorts/r0DFTP6V-cY)</t>
         </is>
       </c>
     </row>
@@ -2981,25 +2981,25 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Interview Warmup by Google</t>
+          <t>ChatGPT</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>https://grow.google/certificates/interview-warmup/</t>
+          <t>https://chatgpt.com</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Practice answering tech and job interview questions with real-time AI transcription and tips.</t>
+          <t>Is website se ye sab kar sakte hain: Conversational AI assistant by OpenAI for answering questions, coding, research, writing, and problem solving. (Channel me kul 18 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Interview candidates with AI (https://www.youtube.com/shorts/SYVGhej9N5M)</t>
+          <t>18 videos (Primary: https://www.youtube.com/shorts/zH8v_47Faw0)</t>
         </is>
       </c>
     </row>
@@ -3011,25 +3011,25 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Toolify.ai</t>
+          <t>Coze AI</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>https://toolify.ai</t>
+          <t>https://coze.com</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: The world's most comprehensive directory of new AI tools, apps, and software updated daily. • AI features: Create both 2D and 3D maps of any place in the world • AI features: Instantly turn your sketch into 3D models • AI features: Create 3D models just by text (Channel me kul 171 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: All-in-one AI bot creation platform powered by GPT-4 and advanced plugins for free.</t>
         </is>
       </c>
       <c r="E85" s="4" t="n">
-        <v>171</v>
+        <v>1</v>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>171 videos (Primary: https://www.youtube.com/shorts/UxLJ7ceAODU)</t>
+          <t>Use ChatGPT for free (https://www.youtube.com/shorts/RgsWlLhZ7V0)</t>
         </is>
       </c>
     </row>
@@ -3041,23 +3041,143 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
+          <t>Flair.ai</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>https://flair.ai</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Is website se ye kar sakte hain: AI product photography studio generating high-end commercial photo shoots in seconds.</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>AI create multiple product images (https://www.youtube.com/shorts/9QpXxmx_HFY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="24" customHeight="1">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>🤖 AI &amp; Machine Learning Tools</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>InVideo AI</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>https://invideo.io</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>Is website se ye kar sakte hain: Full text-to-video AI generator that creates complete edited shorts with voiceovers. (Channel me kul 2 alag-alag videos me featured)</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>2 videos (Primary: https://www.youtube.com/shorts/f6dw_9E-6ss)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="24" customHeight="1">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>🤖 AI &amp; Machine Learning Tools</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>InstantID</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/InstantID/InstantID</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Is website se ye kar sakte hain: State-of-the-art zero-shot identity-preserving image synthesis method.</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Instant ID (https://www.youtube.com/shorts/VGvqzzW4OZc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="24" customHeight="1">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>🤖 AI &amp; Machine Learning Tools</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>Toolify.ai</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>https://toolify.ai</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>Is website se ye sab kar sakte hain: Comprehensive global directory and discovery engine indexing 10,000+ AI software tools, models, and apps updated daily. (Channel me kul 135 alag-alag videos me featured)</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="n">
+        <v>135</v>
+      </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>135 videos (Primary: https://www.youtube.com/shorts/UxLJ7ceAODU)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="24" customHeight="1">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>🤖 AI &amp; Machine Learning Tools</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
           <t>Writesonic</t>
         </is>
       </c>
-      <c r="C86" s="3" t="inlineStr">
+      <c r="C90" s="3" t="inlineStr">
         <is>
           <t>https://writesonic.com</t>
         </is>
       </c>
-      <c r="D86" s="2" t="inlineStr">
+      <c r="D90" s="2" t="inlineStr">
         <is>
           <t>Is website se ye kar sakte hain: AI content writer, SEO article generator, and AI agent platform.</t>
         </is>
       </c>
-      <c r="E86" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F86" s="2" t="inlineStr">
+      <c r="E90" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
         <is>
           <t>Better than ChatGPT for professional article writing (https://www.youtube.com/shorts/29PxGqIq-g4)</t>
         </is>
@@ -3150,6 +3270,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId89"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>